<commit_message>
feat: refactorización de seguridad, implementación de JWT y corrección de histórico
</commit_message>
<xml_diff>
--- a/Copia de Formato_Informe-avance-TIC_Entregable 1.xlsx
+++ b/Copia de Formato_Informe-avance-TIC_Entregable 1.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1e64b9c38bf0dbe8/Desktop/TIC/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C11D7EDC-62FF-4958-B54D-0867BF4D4D92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="8" documentId="8_{C11D7EDC-62FF-4958-B54D-0867BF4D4D92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8B4228D7-774C-4808-9BC0-164FF39B5E23}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="56">
   <si>
     <t>Departamento</t>
   </si>
@@ -153,12 +153,6 @@
 Fecha establecida: 20 de julio, 2026</t>
   </si>
   <si>
-    <t>20 de mayo del 2026</t>
-  </si>
-  <si>
-    <t>Primero</t>
-  </si>
-  <si>
     <t>Sistema IoT para el monitoreo inteligente de la calidad del aire en zonas urbanas de Quito.</t>
   </si>
   <si>
@@ -177,15 +171,9 @@
     <t>15/3/2026</t>
   </si>
   <si>
-    <t>Completo, se corrigió los casos de uso graficados.</t>
-  </si>
-  <si>
     <t>30/5/2026</t>
   </si>
   <si>
-    <t>Redactar la documentación técnica del despliegue en AWS, InfluxDB y Render.</t>
-  </si>
-  <si>
     <t>30/6/2026</t>
   </si>
   <si>
@@ -214,6 +202,12 @@
   </si>
   <si>
     <t>Se mantiene la acción de implementar lógica de reconexión automática en el firmware del ESP32 para las pruebas físicas de campo.</t>
+  </si>
+  <si>
+    <t>5 de julio del 2026</t>
+  </si>
+  <si>
+    <t>Segundo</t>
   </si>
 </sst>
 </file>
@@ -693,6 +687,78 @@
     <xf numFmtId="49" fontId="3" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -700,15 +766,6 @@
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -729,71 +786,8 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1218,59 +1212,59 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="54" customHeight="1" thickBot="1">
-      <c r="A1" s="37" t="s">
+      <c r="A1" s="58" t="s">
         <v>35</v>
       </c>
-      <c r="B1" s="38"/>
-      <c r="C1" s="38"/>
-      <c r="D1" s="38"/>
-      <c r="E1" s="38"/>
+      <c r="B1" s="59"/>
+      <c r="C1" s="59"/>
+      <c r="D1" s="59"/>
+      <c r="E1" s="59"/>
     </row>
     <row r="2" spans="1:5" ht="30">
       <c r="A2" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="44" t="s">
-        <v>37</v>
-      </c>
-      <c r="C2" s="44"/>
+      <c r="B2" s="62" t="s">
+        <v>54</v>
+      </c>
+      <c r="C2" s="62"/>
       <c r="D2" s="27" t="s">
         <v>14</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>38</v>
+        <v>55</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="35.25" customHeight="1">
       <c r="A3" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="B3" s="39" t="s">
-        <v>39</v>
-      </c>
-      <c r="C3" s="39"/>
-      <c r="D3" s="39"/>
-      <c r="E3" s="40"/>
+      <c r="B3" s="60" t="s">
+        <v>37</v>
+      </c>
+      <c r="C3" s="60"/>
+      <c r="D3" s="60"/>
+      <c r="E3" s="61"/>
     </row>
     <row r="4" spans="1:5" ht="15">
       <c r="A4" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B4" s="41" t="s">
-        <v>40</v>
-      </c>
-      <c r="C4" s="42"/>
-      <c r="D4" s="42"/>
-      <c r="E4" s="43"/>
+      <c r="B4" s="36" t="s">
+        <v>38</v>
+      </c>
+      <c r="C4" s="34"/>
+      <c r="D4" s="34"/>
+      <c r="E4" s="37"/>
     </row>
     <row r="5" spans="1:5" ht="28.5">
       <c r="A5" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="39" t="s">
-        <v>41</v>
-      </c>
-      <c r="C5" s="39"/>
+      <c r="B5" s="60" t="s">
+        <v>39</v>
+      </c>
+      <c r="C5" s="60"/>
       <c r="D5" s="7" t="s">
         <v>0</v>
       </c>
@@ -1284,13 +1278,13 @@
       <c r="E6" s="10"/>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="32" t="s">
+      <c r="A7" s="38" t="s">
         <v>27</v>
       </c>
-      <c r="B7" s="33"/>
-      <c r="C7" s="33"/>
-      <c r="D7" s="33"/>
-      <c r="E7" s="34"/>
+      <c r="B7" s="39"/>
+      <c r="C7" s="39"/>
+      <c r="D7" s="39"/>
+      <c r="E7" s="40"/>
     </row>
     <row r="8" spans="1:5" ht="82.5" customHeight="1">
       <c r="A8" s="11" t="s">
@@ -1323,7 +1317,7 @@
         <v>45669</v>
       </c>
       <c r="E9" s="17" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="39" customHeight="1">
@@ -1337,7 +1331,7 @@
         <v>1</v>
       </c>
       <c r="D10" s="19" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="E10" s="17" t="s">
         <v>34</v>
@@ -1354,10 +1348,10 @@
         <v>0.6</v>
       </c>
       <c r="D11" s="19" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="E11" s="28" t="s">
-        <v>45</v>
+        <v>34</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="63" customHeight="1">
@@ -1365,16 +1359,16 @@
         <v>21</v>
       </c>
       <c r="B12" s="15">
-        <v>0.85</v>
+        <v>1</v>
       </c>
       <c r="C12" s="15">
-        <v>0.7</v>
+        <v>1</v>
       </c>
       <c r="D12" s="19" t="s">
-        <v>46</v>
-      </c>
-      <c r="E12" s="62" t="s">
-        <v>47</v>
+        <v>43</v>
+      </c>
+      <c r="E12" s="29" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="68.25" customHeight="1">
@@ -1382,16 +1376,16 @@
         <v>22</v>
       </c>
       <c r="B13" s="15">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="C13" s="15">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="D13" s="19" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="E13" s="28" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="18.95" customHeight="1">
@@ -1405,7 +1399,7 @@
         <v>0</v>
       </c>
       <c r="D14" s="19" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="E14" s="17"/>
     </row>
@@ -1424,98 +1418,98 @@
       <c r="E16" s="17"/>
     </row>
     <row r="17" spans="1:5" ht="14.25" customHeight="1">
-      <c r="A17" s="32" t="s">
+      <c r="A17" s="38" t="s">
         <v>7</v>
       </c>
-      <c r="B17" s="33"/>
-      <c r="C17" s="33"/>
-      <c r="D17" s="33"/>
-      <c r="E17" s="34"/>
+      <c r="B17" s="39"/>
+      <c r="C17" s="39"/>
+      <c r="D17" s="39"/>
+      <c r="E17" s="40"/>
     </row>
     <row r="18" spans="1:5">
-      <c r="A18" s="29" t="s">
+      <c r="A18" s="53" t="s">
         <v>5</v>
       </c>
-      <c r="B18" s="30"/>
-      <c r="C18" s="31"/>
-      <c r="D18" s="35" t="s">
+      <c r="B18" s="54"/>
+      <c r="C18" s="55"/>
+      <c r="D18" s="56" t="s">
         <v>6</v>
       </c>
-      <c r="E18" s="36"/>
+      <c r="E18" s="57"/>
     </row>
     <row r="19" spans="1:5" ht="70.5" customHeight="1">
-      <c r="A19" s="48" t="s">
+      <c r="A19" s="33" t="s">
+        <v>46</v>
+      </c>
+      <c r="B19" s="34"/>
+      <c r="C19" s="35"/>
+      <c r="D19" s="36" t="s">
+        <v>47</v>
+      </c>
+      <c r="E19" s="37"/>
+    </row>
+    <row r="20" spans="1:5" ht="46.9" customHeight="1">
+      <c r="A20" s="33" t="s">
+        <v>48</v>
+      </c>
+      <c r="B20" s="34"/>
+      <c r="C20" s="35"/>
+      <c r="D20" s="36" t="s">
+        <v>49</v>
+      </c>
+      <c r="E20" s="37"/>
+    </row>
+    <row r="21" spans="1:5" ht="59.25" customHeight="1">
+      <c r="A21" s="33" t="s">
         <v>50</v>
       </c>
-      <c r="B19" s="42"/>
-      <c r="C19" s="49"/>
-      <c r="D19" s="41" t="s">
+      <c r="B21" s="34"/>
+      <c r="C21" s="35"/>
+      <c r="D21" s="36" t="s">
         <v>51</v>
       </c>
-      <c r="E19" s="43"/>
-    </row>
-    <row r="20" spans="1:5" ht="46.9" customHeight="1">
-      <c r="A20" s="48" t="s">
+      <c r="E21" s="37"/>
+    </row>
+    <row r="22" spans="1:5" ht="50.25" customHeight="1">
+      <c r="A22" s="33" t="s">
         <v>52</v>
       </c>
-      <c r="B20" s="42"/>
-      <c r="C20" s="49"/>
-      <c r="D20" s="41" t="s">
+      <c r="B22" s="34"/>
+      <c r="C22" s="35"/>
+      <c r="D22" s="36" t="s">
         <v>53</v>
       </c>
-      <c r="E20" s="43"/>
-    </row>
-    <row r="21" spans="1:5" ht="59.25" customHeight="1">
-      <c r="A21" s="48" t="s">
-        <v>54</v>
-      </c>
-      <c r="B21" s="42"/>
-      <c r="C21" s="49"/>
-      <c r="D21" s="41" t="s">
-        <v>55</v>
-      </c>
-      <c r="E21" s="43"/>
-    </row>
-    <row r="22" spans="1:5" ht="50.25" customHeight="1">
-      <c r="A22" s="48" t="s">
-        <v>56</v>
-      </c>
-      <c r="B22" s="42"/>
-      <c r="C22" s="49"/>
-      <c r="D22" s="41" t="s">
-        <v>57</v>
-      </c>
-      <c r="E22" s="43"/>
+      <c r="E22" s="37"/>
     </row>
     <row r="23" spans="1:5">
-      <c r="A23" s="48"/>
-      <c r="B23" s="42"/>
-      <c r="C23" s="49"/>
-      <c r="D23" s="41"/>
-      <c r="E23" s="43"/>
+      <c r="A23" s="33"/>
+      <c r="B23" s="34"/>
+      <c r="C23" s="35"/>
+      <c r="D23" s="36"/>
+      <c r="E23" s="37"/>
     </row>
     <row r="24" spans="1:5">
-      <c r="A24" s="32" t="s">
+      <c r="A24" s="38" t="s">
         <v>28</v>
       </c>
-      <c r="B24" s="33"/>
-      <c r="C24" s="33"/>
-      <c r="D24" s="33"/>
-      <c r="E24" s="34"/>
+      <c r="B24" s="39"/>
+      <c r="C24" s="39"/>
+      <c r="D24" s="39"/>
+      <c r="E24" s="40"/>
     </row>
     <row r="25" spans="1:5">
-      <c r="A25" s="50"/>
-      <c r="B25" s="51"/>
-      <c r="C25" s="52"/>
+      <c r="A25" s="41"/>
+      <c r="B25" s="42"/>
+      <c r="C25" s="43"/>
       <c r="D25" s="20"/>
       <c r="E25" s="21"/>
     </row>
     <row r="26" spans="1:5" ht="36" customHeight="1">
-      <c r="A26" s="53" t="s">
+      <c r="A26" s="44" t="s">
         <v>36</v>
       </c>
-      <c r="B26" s="54"/>
-      <c r="C26" s="55"/>
+      <c r="B26" s="45"/>
+      <c r="C26" s="46"/>
       <c r="D26" s="22" t="s">
         <v>19</v>
       </c>
@@ -1524,9 +1518,9 @@
       </c>
     </row>
     <row r="27" spans="1:5" ht="29.1" customHeight="1">
-      <c r="A27" s="56"/>
-      <c r="B27" s="57"/>
-      <c r="C27" s="58"/>
+      <c r="A27" s="47"/>
+      <c r="B27" s="48"/>
+      <c r="C27" s="49"/>
       <c r="D27" s="1" t="s">
         <v>8</v>
       </c>
@@ -1535,9 +1529,9 @@
       </c>
     </row>
     <row r="28" spans="1:5" ht="24" customHeight="1">
-      <c r="A28" s="59"/>
-      <c r="B28" s="60"/>
-      <c r="C28" s="61"/>
+      <c r="A28" s="50"/>
+      <c r="B28" s="51"/>
+      <c r="C28" s="52"/>
       <c r="D28" s="25" t="s">
         <v>9</v>
       </c>
@@ -1546,13 +1540,13 @@
       </c>
     </row>
     <row r="29" spans="1:5" ht="98.1" customHeight="1" thickBot="1">
-      <c r="A29" s="45" t="s">
+      <c r="A29" s="30" t="s">
         <v>29</v>
       </c>
-      <c r="B29" s="46"/>
-      <c r="C29" s="46"/>
-      <c r="D29" s="46"/>
-      <c r="E29" s="47"/>
+      <c r="B29" s="31"/>
+      <c r="C29" s="31"/>
+      <c r="D29" s="31"/>
+      <c r="E29" s="32"/>
     </row>
     <row r="30" spans="1:5" ht="51.95" customHeight="1">
       <c r="A30" s="1"/>
@@ -1586,6 +1580,15 @@
     </row>
   </sheetData>
   <mergeCells count="23">
+    <mergeCell ref="A18:C18"/>
+    <mergeCell ref="A17:E17"/>
+    <mergeCell ref="A7:E7"/>
+    <mergeCell ref="D18:E18"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="B3:E3"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B4:E4"/>
+    <mergeCell ref="B2:C2"/>
     <mergeCell ref="A29:E29"/>
     <mergeCell ref="A19:C19"/>
     <mergeCell ref="A20:C20"/>
@@ -1600,15 +1603,6 @@
     <mergeCell ref="A26:C28"/>
     <mergeCell ref="D19:E19"/>
     <mergeCell ref="D20:E20"/>
-    <mergeCell ref="A18:C18"/>
-    <mergeCell ref="A17:E17"/>
-    <mergeCell ref="A7:E7"/>
-    <mergeCell ref="D18:E18"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="B3:E3"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="B4:E4"/>
-    <mergeCell ref="B2:C2"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.79000000000000015" right="0.79000000000000015" top="1.18" bottom="0.79000000000000015" header="0.39000000000000007" footer="0.30000000000000004"/>

</xml_diff>